<commit_message>
Fix customer-facing content tone and Excel header color
- content_suite_prompts: clarify that "sếp" tone applies only to AI↔owner comms, post content addressing end customers must use "bạn/anh chị"
- content_suite_prompts: fix hook angle example "Sếp đã từng [pain]?" → "Bạn đã từng [pain]?" (appeared in 2 prompts)
- content_suite_prompts: fix CTA example that used "sếp" for end customer
- renderers.py: tone down Excel header fill 2563EB (bright blue) → 2C3E50 (dark navy)
- gen_sample_content.py: replace all customer-addressing "sếp" → "bạn" in social post mock data

https://claude.ai/code/session_01VCiaeRtCx7WsxWpgX47rVx
</commit_message>
<xml_diff>
--- a/sample_lotus_social_posts.xlsx
+++ b/sample_lotus_social_posts.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="G4" s="29" t="inlineStr">
         <is>
-          <t>Mùa đông da thường bị mất nước nhiều hơn bạn nghĩ — không phải vì không dưỡng ẩm, mà vì dưỡng ẩm sai thứ tự. Đây là 3 điều Lotus hay gặp nhất ở khách đến lần đầu: 1. Dùng serum trước toner (khóa ẩm sai lớp) / 2. Bỏ qua dầu dưỡng — lớp "khóa" quan trọng nhất mùa lạnh / 3. Rửa mặt nước quá nóng — phá vỡ hàng rào bảo vệ da. Mùa này da cần được giữ ấm từ bên trong, không chỉ thoa kem bên ngoài. Đông y có cách nhìn khác: da khô mùa đông thường liên quan đến tình trạng thiếu huyết khí — bổ từ bên trong mới giải quyết gốc rễ. Sếp đang gặp vấn đề gì với da mùa này?</t>
+          <t>Mùa đông da thường bị mất nước nhiều hơn bạn nghĩ — không phải vì không dưỡng ẩm, mà vì dưỡng ẩm sai thứ tự. Đây là 3 điều Lotus hay gặp nhất ở khách đến lần đầu: 1. Dùng serum trước toner (khóa ẩm sai lớp) / 2. Bỏ qua dầu dưỡng — lớp "khóa" quan trọng nhất mùa lạnh / 3. Rửa mặt nước quá nóng — phá vỡ hàng rào bảo vệ da. Mùa này da cần được giữ ấm từ bên trong, không chỉ thoa kem bên ngoài. Đông y có cách nhìn khác: da khô mùa đông thường liên quan đến tình trạng thiếu huyết khí — bổ từ bên trong mới giải quyết gốc rễ. Bạn đang gặp vấn đề gì với da mùa này?</t>
         </is>
       </c>
       <c r="H4" s="29" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="G6" s="29" t="inlineStr">
         <is>
-          <t>Da mùa đông — mỗi người một kiểu khổ khác nhau. Có người khô bong tróc dù thoa kem liên tục. Có người nổi mụn ẩn hàng loạt dù không ăn gì lạ. Có người nám tối hơn hẳn dù không ra nắng. Có người da căng rát như bị kéo, đặc biệt sau khi rửa mặt. Em hỏi vì muốn hiểu sếp đang gặp vấn đề gì thật sự — không phải để bán, mà để chia sẻ đúng thứ sếp cần. Tuần này em sẽ trả lời từng comment cụ thể. Không copy-paste, không tư vấn chung chung.</t>
+          <t>Da mùa đông — mỗi người một kiểu khổ khác nhau. Có người khô bong tróc dù thoa kem liên tục. Có người nổi mụn ẩn hàng loạt dù không ăn gì lạ. Có người nám tối hơn hẳn dù không ra nắng. Có người da căng rát như bị kéo, đặc biệt sau khi rửa mặt. Em hỏi vì muốn hiểu bạn đang gặp vấn đề gì thật sự — không phải để bán, mà để chia sẻ đúng thứ bạn cần. Tuần này em sẽ trả lời từng comment cụ thể. Không copy-paste, không tư vấn chung chung.</t>
         </is>
       </c>
       <c r="H6" s="29" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="G7" s="31" t="inlineStr">
         <is>
-          <t>Có một sự thật brand không bao giờ nói với bạn: 80% hiệu quả của skincare đến từ CÁCH dùng, không phải sản phẩm. Serum đắt tiền mà layer sai thứ tự — uổng. Kem chống nắng tốt mà thoa không đủ lượng — không bảo vệ được. Retinol xịn mà dùng ban ngày — hại da. Đông y có nguyên tắc tương tự: thảo dược quý đến đâu, sắc sai cách hoặc uống sai giờ — không hiệu quả, thậm chí phản tác dụng. Dưới đây là 5 lỗi sai phổ biến nhất em gặp khi tư vấn khách — không phân biệt skincare rẻ hay đắt: 1. Dùng AHA/BHA cùng Vitamin C buổi sáng / 2. Thoa retinol trên da ẩm (tăng kích ứng) / 3. Bỏ qua toner trước serum / 4. Thoa SPF quá mỏng — cần 2 ngón tay mới đủ / 5. Mix quá nhiều active cùng lúc. Sếp đang mắc lỗi nào không?</t>
+          <t>Có một sự thật brand không bao giờ nói với bạn: 80% hiệu quả của skincare đến từ CÁCH dùng, không phải sản phẩm. Serum đắt tiền mà layer sai thứ tự — uổng. Kem chống nắng tốt mà thoa không đủ lượng — không bảo vệ được. Retinol xịn mà dùng ban ngày — hại da. Đông y có nguyên tắc tương tự: thảo dược quý đến đâu, sắc sai cách hoặc uống sai giờ — không hiệu quả, thậm chí phản tác dụng. Dưới đây là 5 lỗi sai phổ biến nhất em gặp khi tư vấn khách — không phân biệt skincare rẻ hay đắt: 1. Dùng AHA/BHA cùng Vitamin C buổi sáng / 2. Thoa retinol trên da ẩm (tăng kích ứng) / 3. Bỏ qua toner trước serum / 4. Thoa SPF quá mỏng — cần 2 ngón tay mới đủ / 5. Mix quá nhiều active cùng lúc. Bạn đang mắc lỗi nào không?</t>
         </is>
       </c>
       <c r="H7" s="31" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="F9" s="31" t="inlineStr">
         <is>
-          <t>"Quy trình 5 bước tại Lotus Spa — em chia sẻ để sếp hiểu mình đang làm gì với da của mình."</t>
+          <t>"Quy trình 5 bước tại Lotus Spa — em chia sẻ để bạn hiểu mình đang làm gì với da của mình."</t>
         </is>
       </c>
       <c r="G9" s="31" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="G10" s="29" t="inlineStr">
         <is>
-          <t>Em hiểu câu hỏi này — vì ai cũng đã từng bỏ tiền mà không thấy kết quả. Câu trả lời trung thực: Tùy vấn đề và tạng thể của mỗi người. Nhưng em có thể nói cụ thể hơn: Da thường (chăm sóc cơ bản): 2-3 buổi thấy da mịn, sáng hơn. Nám nhẹ (mới xuất hiện dưới 1 năm): 6-8 buổi thấy nhạt rõ. Nám sâu (trên 2-3 năm, đã laser): 12-16 buổi, kết hợp điều chỉnh nội tiết. Mụn viêm cấp: 3-4 buổi giảm viêm, 8-10 buổi ổn định. Em không hứa kết quả cụ thể vì mỗi người một tạng thể. Nhưng em hứa: sau buổi đầu tiên sếp sẽ biết mình phù hợp không, trước khi quyết định gói dài.</t>
+          <t>Em hiểu câu hỏi này — vì ai cũng đã từng bỏ tiền mà không thấy kết quả. Câu trả lời trung thực: Tùy vấn đề và tạng thể của mỗi người. Nhưng em có thể nói cụ thể hơn: Da thường (chăm sóc cơ bản): 2-3 buổi thấy da mịn, sáng hơn. Nám nhẹ (mới xuất hiện dưới 1 năm): 6-8 buổi thấy nhạt rõ. Nám sâu (trên 2-3 năm, đã laser): 12-16 buổi, kết hợp điều chỉnh nội tiết. Mụn viêm cấp: 3-4 buổi giảm viêm, 8-10 buổi ổn định. Em không hứa kết quả cụ thể vì mỗi người một tạng thể. Nhưng em hứa: sau buổi đầu tiên bạn sẽ biết mình phù hợp không, trước khi quyết định gói dài.</t>
         </is>
       </c>
       <c r="H10" s="29" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="G11" s="31" t="inlineStr">
         <is>
-          <t>[REPOST VIDEO TIKTOK CỦA KHÁCH] Em không dàn dựng, không nhờ quay, không trả thù lao. Chị tự quay, tự đăng, tự tag Lotus. Đây là loại review em trân trọng nhất — vì nó thật. Nếu sếp đang phân vân có nên thử Lotus không, có thể inbox em để nghe thêm từ những khách đang điều trị. Em sẵn sàng kết nối — không phải để thuyết phục, mà để sếp có đủ thông tin quyết định.</t>
+          <t>[REPOST VIDEO TIKTOK CỦA KHÁCH] Em không dàn dựng, không nhờ quay, không trả thù lao. Chị tự quay, tự đăng, tự tag Lotus. Đây là loại review em trân trọng nhất — vì nó thật. Nếu bạn đang phân vân có nên thử Lotus không, có thể inbox em để nghe thêm từ những khách đang điều trị. Em sẵn sàng kết nối — không phải để thuyết phục, mà để bạn có đủ thông tin quyết định.</t>
         </is>
       </c>
       <c r="H11" s="31" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="G12" s="29" t="inlineStr">
         <is>
-          <t>Lotus không hay làm flash sale. Lần này em quyết định vì 1 lý do: Tết là thời điểm nhiều sếp muốn "reset" da trước khi về nhà, trước khi gặp họ hàng, trước khi chụp ảnh Tết. Em hiểu cảm giác đó. Combo Tết 680K bao gồm: 1 buổi thăm khám + phân loại tạng thể (trị giá 150K) / 1 liệu trình trị liệu Đông y 90 phút (trị giá 450K) / 1 set hướng dẫn skincare tại nhà theo tạng thể (trị giá 250K). Tổng thật: 850K. Em giảm còn 680K — tiết kiệm 170K. Tại sao 10 slot? Vì mỗi buổi thăm khám mất 20 phút, em chỉ có thể nhận 10 ca mới trong tháng mà vẫn đảm bảo chất lượng cho khách cũ. Không phải chiêu marketing. Là giới hạn thật của lịch em.</t>
+          <t>Lotus không hay làm flash sale. Lần này em quyết định vì 1 lý do: Tết là thời điểm nhiều bạn muốn "reset" da trước khi về nhà, trước khi gặp họ hàng, trước khi chụp ảnh Tết. Em hiểu cảm giác đó. Combo Tết 680K bao gồm: 1 buổi thăm khám + phân loại tạng thể (trị giá 150K) / 1 liệu trình trị liệu Đông y 90 phút (trị giá 450K) / 1 set hướng dẫn skincare tại nhà theo tạng thể (trị giá 250K). Tổng thật: 850K. Em giảm còn 680K — tiết kiệm 170K. Tại sao 10 slot? Vì mỗi buổi thăm khám mất 20 phút, em chỉ có thể nhận 10 ca mới trong tháng mà vẫn đảm bảo chất lượng cho khách cũ. Không phải chiêu marketing. Là giới hạn thật của lịch em.</t>
         </is>
       </c>
       <c r="H12" s="29" t="inlineStr">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="G13" s="31" t="inlineStr">
         <is>
-          <t>Với những sếp đã đồng hành cùng Lotus từ năm 2021, 2022 — em muốn nói thẳng: Năm nay Lotus sẽ ưu tiên giữ slot cho các sếp cũ trước khi nhận khách mới. Đây không phải thông báo marketing — đây là cam kết em giữ từ ngày mở. Sếp nào cần đặt lịch Tết (20/01 - 28/01), inbox em trước 22/01 — em sắp xếp ưu tiên. Không cần combo, không cần deal. Chỉ cần nhắn "đặt lịch" là em lo. Cảm ơn sếp đã tin Lotus trong những năm qua. Mỗi case sếp chia sẻ với em đều là bài học em mang theo.</t>
+          <t>Với những ai đã đồng hành cùng Lotus từ năm 2021, 2022 — em muốn nói thẳng: Năm nay Lotus sẽ ưu tiên giữ slot cho các khách cũ trước khi nhận khách mới. Đây không phải thông báo marketing — đây là cam kết em giữ từ ngày mở. Ai cần đặt lịch Tết (20/01 - 28/01), inbox em trước 22/01 — em sắp xếp ưu tiên. Không cần combo, không cần deal. Chỉ cần nhắn "đặt lịch" là em lo. Cảm ơn bạn đã tin Lotus trong những năm qua. Mỗi case bạn chia sẻ với em đều là bài học em mang theo.</t>
         </is>
       </c>
       <c r="H13" s="31" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="G14" s="29" t="inlineStr">
         <is>
-          <t>Em không muốn tạo urgency giả. Đây là thật: Hôm nay 26/01. Lotus đóng cửa nghỉ Tết từ 29/01. Còn đúng 5 slot combo Tết 680K chưa có người đặt. Sau 28/01, em không nhận thêm — không phải vì hết deal, mà vì em cần chuẩn bị cho lịch tháng 2 của khách cũ. Nếu sếp đang phân vân từ hồi đầu tháng mà chưa quyết: đây là lần cuối em nhắc. Không inbox sau 28/01 thì xem lịch tháng 2 nhé.</t>
+          <t>Em không muốn tạo urgency giả. Đây là thật: Hôm nay 26/01. Lotus đóng cửa nghỉ Tết từ 29/01. Còn đúng 5 slot combo Tết 680K chưa có người đặt. Sau 28/01, em không nhận thêm — không phải vì hết deal, mà vì em cần chuẩn bị cho lịch tháng 2 của khách cũ. Nếu bạn đang phân vân từ hồi đầu tháng mà chưa quyết: đây là lần cuối em nhắc. Không inbox sau 28/01 thì xem lịch tháng 2 nhé.</t>
         </is>
       </c>
       <c r="H14" s="29" t="inlineStr">
@@ -1545,12 +1545,12 @@
       </c>
       <c r="F15" s="31" t="inlineStr">
         <is>
-          <t>"Tháng 1 của Lotus kết thúc ở đây — cảm ơn sếp đã cùng em đi qua 28 ngày này."</t>
+          <t>"Tháng 1 của Lotus kết thúc ở đây — cảm ơn bạn đã cùng em đi qua 28 ngày này."</t>
         </is>
       </c>
       <c r="G15" s="31" t="inlineStr">
         <is>
-          <t>Tháng 1/2026 — Lotus phục vụ 47 khách. 12 ca mới, 35 ca tái khám. 3 ca nám đã kết thúc liệu trình, đang duy trì. 1 ca viêm da cơ địa lần đầu tiên ngủ ngon sau 2 năm. 2 ca trị mụn nội tiết thấy chu kỳ ổn định lại. Em không đăng số để khoe. Em đăng để nhớ. Mỗi con số là 1 người thật, 1 câu chuyện thật, 1 buổi sáng ngủ dậy nhìn gương và thấy mình khác đi. Tháng 2 Lotus mở lịch từ 03/02 sau Tết. Sếp nào muốn đặt lịch sớm — inbox em trước 30/01 để ưu tiên giữ slot. Chúc sếp Tết ấm áp. Hẹn gặp lại.</t>
+          <t>Tháng 1/2026 — Lotus phục vụ 47 khách. 12 ca mới, 35 ca tái khám. 3 ca nám đã kết thúc liệu trình, đang duy trì. 1 ca viêm da cơ địa lần đầu tiên ngủ ngon sau 2 năm. 2 ca trị mụn nội tiết thấy chu kỳ ổn định lại. Em không đăng số để khoe. Em đăng để nhớ. Mỗi con số là 1 người thật, 1 câu chuyện thật, 1 buổi sáng ngủ dậy nhìn gương và thấy mình khác đi. Tháng 2 Lotus mở lịch từ 03/02 sau Tết. Ai muốn đặt lịch sớm — inbox em trước 30/01 để ưu tiên giữ slot. Chúc bạn Tết ấm áp. Hẹn gặp lại.</t>
         </is>
       </c>
       <c r="H15" s="31" t="inlineStr">
@@ -1614,17 +1614,17 @@
       </c>
       <c r="F16" s="29" t="inlineStr">
         <is>
-          <t>"Tips chăm da mùa đông từ Lotus — quà đầu năm cho sếp."</t>
+          <t>"Tips chăm da mùa đông từ Lotus — quà đầu năm cho bạn."</t>
         </is>
       </c>
       <c r="G16" s="29" t="inlineStr">
         <is>
-          <t>Đầu năm mới, Lotus gửi sếp 3 tips chăm da mùa đông từ góc nhìn Đông y: 1. Uống nước ấm thay nước lạnh — giúp tỳ vị hấp thụ tốt hơn, da ẩm từ bên trong. 2. Ăn thêm vừng đen + hạt óc chó — bổ thận, nuôi da tóc móng mùa lạnh. 3. Ngủ trước 23h ít nhất 4 ngày/tuần — gan hoạt động 23h-1h sáng, ảnh hưởng trực tiếp đến màu da. Chúc sếp năm mới sức khỏe, da đẹp từ bên trong!</t>
+          <t>Đầu năm mới, Lotus gửi bạn 3 tips chăm da mùa đông từ góc nhìn Đông y: 1. Uống nước ấm thay nước lạnh — giúp tỳ vị hấp thụ tốt hơn, da ẩm từ bên trong. 2. Ăn thêm vừng đen + hạt óc chó — bổ thận, nuôi da tóc móng mùa lạnh. 3. Ngủ trước 23h ít nhất 4 ngày/tuần — gan hoạt động 23h-1h sáng, ảnh hưởng trực tiếp đến màu da. Chúc bạn năm mới sức khỏe, da đẹp từ bên trong!</t>
         </is>
       </c>
       <c r="H16" s="29" t="inlineStr">
         <is>
-          <t>Inbox "TƯ VẤN" nếu sếp muốn em xem da cụ thể</t>
+          <t>Inbox "TƯ VẤN" nếu bạn muốn em xem da cụ thể</t>
         </is>
       </c>
       <c r="I16" s="29" t="inlineStr">
@@ -1683,17 +1683,17 @@
       </c>
       <c r="F17" s="31" t="inlineStr">
         <is>
-          <t>"Lâu rồi chưa gặp sếp — da dạo này thế nào ạ?"</t>
+          <t>"Lâu rồi chưa gặp bạn — da dạo này thế nào ạ?"</t>
         </is>
       </c>
       <c r="G17" s="31" t="inlineStr">
         <is>
-          <t>Dạ em là Lotus Spa. Em thấy sếp chưa quay lại khoảng 2 tháng nay. Không hối thúc — chỉ hỏi thăm thật. Mùa đông này da thường khó hơn, đặc biệt với những vấn đề cần duy trì đều. Nếu sếp đang bận hoặc đang thử cách khác thì hoàn toàn OK. Nếu sếp muốn check lại tình trạng da, Lotus có slot tuần này. Không cần đặt gói mới — em xem lại và tư vấn tiếp theo tình trạng hiện tại của sếp thôi.</t>
+          <t>Dạ em là Lotus Spa. Em thấy bạn chưa quay lại khoảng 2 tháng nay. Không hối thúc — chỉ hỏi thăm thật. Mùa đông này da thường khó hơn, đặc biệt với những vấn đề cần duy trì đều. Nếu bạn đang bận hoặc đang thử cách khác thì hoàn toàn OK. Nếu bạn muốn check lại tình trạng da, Lotus có slot tuần này. Không cần đặt gói mới — em xem lại và tư vấn tiếp theo tình trạng hiện tại của bạn thôi.</t>
         </is>
       </c>
       <c r="H17" s="31" t="inlineStr">
         <is>
-          <t>Nhắn "CHECK DA" để em đặt lịch cho sếp</t>
+          <t>Nhắn "CHECK DA" để em đặt lịch cho bạn</t>
         </is>
       </c>
       <c r="I17" s="31" t="inlineStr"/>
@@ -1748,12 +1748,12 @@
       </c>
       <c r="F18" s="29" t="inlineStr">
         <is>
-          <t>"Sếp ơi — combo Tết 680K, Lotus ưu tiên báo khách cũ trước."</t>
+          <t>"Bạn ơi — combo Tết 680K, Lotus ưu tiên báo khách cũ trước."</t>
         </is>
       </c>
       <c r="G18" s="29" t="inlineStr">
         <is>
-          <t>Dạ Lotus đang có combo trước Tết: 1 buổi thăm khám + liệu trình Đông y 90 phút + hướng dẫn skincare tại nhà — 680K (gốc 850K). Sếp là khách cũ nên em báo trước khi đăng công khai. Còn 8 slot, ưu tiên đặt trước 22/01. Sếp nhắn "ĐẶT LỊCH" là em confirm ngay ạ.</t>
+          <t>Dạ Lotus đang có combo trước Tết: 1 buổi thăm khám + liệu trình Đông y 90 phút + hướng dẫn skincare tại nhà — 680K (gốc 850K). Bạn là khách cũ nên em báo trước khi đăng công khai. Còn 8 slot, ưu tiên đặt trước 22/01. Bạn nhắn "ĐẶT LỊCH" là em confirm ngay ạ.</t>
         </is>
       </c>
       <c r="H18" s="29" t="inlineStr">
@@ -1813,12 +1813,12 @@
       </c>
       <c r="F19" s="31" t="inlineStr">
         <is>
-          <t>"Lotus nghỉ Tết từ 29/01 — cảm ơn sếp năm nay."</t>
+          <t>"Lotus nghỉ Tết từ 29/01 — cảm ơn bạn năm nay."</t>
         </is>
       </c>
       <c r="G19" s="31" t="inlineStr">
         <is>
-          <t>Dạ Lotus nghỉ Tết từ ngày mai 29/01, mở cửa trở lại 03/02 ạ. Cảm ơn sếp đã tin tưởng Lotus trong năm 2025. Mỗi lần sếp ghé là thêm 1 kỷ niệm em trân trọng. Chúc sếp Tết ấm áp, vui vẻ bên gia đình. Sức khỏe, bình an, và da đẹp từ bên trong nhé sếp! Hẹn gặp lại tháng 2.</t>
+          <t>Dạ Lotus nghỉ Tết từ ngày mai 29/01, mở cửa trở lại 03/02 ạ. Cảm ơn bạn đã tin tưởng Lotus trong năm 2025. Mỗi lần bạn ghé là thêm 1 kỷ niệm em trân trọng. Chúc bạn Tết ấm áp, vui vẻ bên gia đình. Sức khỏe, bình an, và da đẹp từ bên trong nhé bạn! Hẹn gặp lại tháng 2.</t>
         </is>
       </c>
       <c r="H19" s="31" t="inlineStr"/>

</xml_diff>